<commit_message>
Remove Comment out code and Add D column formulas and add Step 9
</commit_message>
<xml_diff>
--- a/Company Code Mapping.xlsx
+++ b/Company Code Mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f11c2d5f9d09f2b0/Desktop/company 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{B4043AC5-FEE7-4DF6-8E06-8AAE81C9CA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C858946-1A17-4ABB-B7C2-D4C9DCA1C505}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{B4043AC5-FEE7-4DF6-8E06-8AAE81C9CA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A442987-5CF0-4494-A3F7-471B78D8E83A}"/>
   <bookViews>
     <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" xr2:uid="{62802EC6-B32D-478B-93BD-BFB9F05E93D8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="144">
   <si>
     <t>TOTAL AMOUNTS</t>
   </si>
@@ -551,6 +551,9 @@
   </si>
   <si>
     <t>delete</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -1404,10 +1407,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1773,11 +1772,11 @@
       </c>
       <c r="D3" s="50">
         <f>SUM(D4:D5)</f>
-        <v>1000000</v>
+        <v>0</v>
       </c>
       <c r="E3" s="51">
         <f>SUM(E4:E5)</f>
-        <v>5000000</v>
+        <v>6000000</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.3" thickBot="1" x14ac:dyDescent="0.35">
@@ -1811,11 +1810,11 @@
       </c>
       <c r="D5" s="54">
         <f>IF(D6="Yes",C5,0)</f>
-        <v>1000000</v>
+        <v>0</v>
       </c>
       <c r="E5" s="55">
         <f>+C5-D5</f>
-        <v>0</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15.65" x14ac:dyDescent="0.3">
@@ -1825,7 +1824,7 @@
       <c r="B6" s="99"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E6" s="11"/>
     </row>
@@ -1939,11 +1938,11 @@
       </c>
       <c r="D13" s="51">
         <f>+D3-D8</f>
-        <v>-166666.66666666674</v>
+        <v>-1166666.6666666667</v>
       </c>
       <c r="E13" s="51">
         <f>+E3-E8</f>
-        <v>3166666.6666666665</v>
+        <v>4166666.6666666665</v>
       </c>
     </row>
     <row r="14" spans="1:6" thickBot="1" x14ac:dyDescent="0.35">
@@ -2167,11 +2166,11 @@
       </c>
       <c r="D26" s="51">
         <f>+D13-D15</f>
-        <v>-2416666.666666667</v>
+        <v>-3416666.666666667</v>
       </c>
       <c r="E26" s="51">
         <f>+E13-E15</f>
-        <v>-8083333.333333334</v>
+        <v>-7083333.333333334</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="15.65" thickBot="1" x14ac:dyDescent="0.35">
@@ -2901,11 +2900,11 @@
       </c>
       <c r="D66" s="51">
         <f>+D26-D28+D56</f>
-        <v>-6916666.6666666679</v>
+        <v>-7916666.6666666679</v>
       </c>
       <c r="E66" s="51">
         <f>+E26-E28+E56</f>
-        <v>-30583333.333333336</v>
+        <v>-29583333.333333336</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="16.3" thickBot="1" x14ac:dyDescent="0.35">
@@ -3663,11 +3662,11 @@
       </c>
       <c r="D108" s="51">
         <f>+D66+D68-D101</f>
-        <v>-2000000.0000000028</v>
+        <v>-3000000.0000000028</v>
       </c>
       <c r="E108" s="51">
         <f>+E66+E68-E101</f>
-        <v>-6000000.0000000037</v>
+        <v>-5000000.0000000037</v>
       </c>
     </row>
     <row r="109" spans="1:6" customFormat="1" ht="15.65" thickBot="1" x14ac:dyDescent="0.35">
@@ -3764,11 +3763,11 @@
       </c>
       <c r="D115" s="88">
         <f>+D108-D110</f>
-        <v>-2750000.0000000028</v>
+        <v>-3750000.0000000028</v>
       </c>
       <c r="E115" s="88">
         <f>+E108-E110</f>
-        <v>-9750000.0000000037</v>
+        <v>-8750000.0000000037</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="16.3" thickBot="1" x14ac:dyDescent="0.35">
@@ -3874,11 +3873,11 @@
       </c>
       <c r="D121" s="30">
         <f>SUM(D115:D120)</f>
-        <v>-2750000.0000000028</v>
+        <v>-3750000.0000000028</v>
       </c>
       <c r="E121" s="30">
         <f>SUM(E115:E120)</f>
-        <v>-9750000.0000000037</v>
+        <v>-8750000.0000000037</v>
       </c>
     </row>
     <row r="122" spans="1:5" customFormat="1" ht="15.65" thickBot="1" x14ac:dyDescent="0.35">
@@ -3934,7 +3933,7 @@
       <c r="D126" s="90"/>
       <c r="E126" s="30">
         <f>+E121-E123</f>
-        <v>-11250000.000000004</v>
+        <v>-10250000.000000004</v>
       </c>
     </row>
     <row r="127" spans="1:5" customFormat="1" ht="15.65" thickBot="1" x14ac:dyDescent="0.35">
@@ -3951,7 +3950,7 @@
       <c r="D128" s="90"/>
       <c r="E128" s="43">
         <f>(MAX(E129,E131,E132)+E130)+E133+E134+E135+E136+E137</f>
-        <v>25000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="16.3" thickBot="1" x14ac:dyDescent="0.35">
@@ -3979,7 +3978,7 @@
       <c r="D130" s="90"/>
       <c r="E130" s="32">
         <f>+D5*0.025</f>
-        <v>25000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="16.3" thickBot="1" x14ac:dyDescent="0.35">
@@ -4079,7 +4078,7 @@
       <c r="D139" s="90"/>
       <c r="E139" s="31">
         <f>SUM(E140:E141)</f>
-        <v>25000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:6" ht="16.3" thickBot="1" x14ac:dyDescent="0.35">
@@ -4107,12 +4106,12 @@
       </c>
       <c r="C141" s="38">
         <f>IF(C142="Yes",E128,"")</f>
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="D141" s="90"/>
       <c r="E141" s="32">
         <f>+C141</f>
-        <v>25000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="15.65" x14ac:dyDescent="0.3">

</xml_diff>